<commit_message>
Update topic news feed
</commit_message>
<xml_diff>
--- a/data/topic_feeds.xlsx
+++ b/data/topic_feeds.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4429,6 +4429,2514 @@
         <v>46013.61065972222</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>US economy grew strongly in third quarter, GDP report says - The Guardian</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 13:41:00 GMT</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPYXBVUXdiVWd3X3hOZk15a1F5MEowd2hkdFJGanYtQ0ZVMERfYVJwMEdPSjJyQXhVMXhWSnFkNGxxTnA2VUxhdzYyQnE1MXZfWmZIMHUzSi15VDZLaXEyemtiM25tQVRXV1dJZklHYW1ENkM5em5ITnRISzBTUS1TZy1ENA?oc=5</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>7</v>
+      </c>
+      <c r="G122" s="2" t="n">
+        <v>46014.57013888889</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>UK Government Urged to Review Palantir Contracts After Swiss Security Report - TechRepublic</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:59:34 GMT</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNTHlMeWFVcUNqVUVqSVhOTzlsT1EzSzJMQ2JKbDdERi0wWUtCTFZxN2FzUXotN0I1ZmdoeDNObTVZZWRaWVFmQ0ZlTnl1RVlERWhxWmt1bHFOLXpUQnppeEt6YkxLT2NPd01VcXFCbGtQZjJoYUJublNwNXRjcUxJNQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>7</v>
+      </c>
+      <c r="G123" s="2" t="n">
+        <v>46014.66636574074</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>CM says Inquiry Report "completely exonerates" the Government - Gibraltar Broadcasting Corporation</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 20:37:30 GMT</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPdC1HV3hmRVNxZkVYRUJZaGFpbUxvcTMyMTlEMlJqT2dDc0NXTHNMZ1RpUlktR3plZ2JSWk1uQnRhZ053UGpVNUs4cXFYZ25IT1ZhVG4zS2dTT2VtQnZocXhPOXp1cW5NZmVnR25xcUhYR2owNTlWLV9sMjBqaW02TnZUeXhkSnhoZ3lR?oc=5</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>7</v>
+      </c>
+      <c r="G124" s="2" t="n">
+        <v>46014.859375</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>iOS 26.3: EU Regulation Forces Apple's Biggest Update - Gadget Hacks</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 14:34:15 GMT</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQdnlhQmpUSDdGZGZGZXFpazV1OGNTSkhSV011VzFRRndEYzlmUnRaa2VPVU9YRTdabGtZNWxBUDlKU25GTFZHYTBBcGNYNGQ3YXlUQ2RVWTNDN3lGLUdGdlY0bTN0eWN5SzF4TTVmZG9XVklDTFdYYUZpYVEwblJlXzluQzZkNUppOGhhMDExMA?oc=5</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>7</v>
+      </c>
+      <c r="G125" s="2" t="n">
+        <v>46014.60711805556</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Ministry of Labour Sets Policy for Public Holidays - Syria Report</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 16:26:26 GMT</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPZG1jTUV0OVVHWVR2Q09kcXBGQ2ZqSVlIY0VRcXlCYjFGTkwxWlpGcml2b0k3aHc2enNDc19uOVBHVU9vWURNcTFhWVhtT0lSWHVQVGw2MldTbXlPZW5odDl1LWh4X1FyUVAtYlJ2TEI1VnUzbG9yWHpOaEtFclp3ZFdB?oc=5</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>7</v>
+      </c>
+      <c r="G126" s="2" t="n">
+        <v>46014.68502314815</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Government provides update on 5% Deposit Scheme - Broker Daily</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:25:00 GMT</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQeWU5YTl6c3F5cW9TWjN2V21HNlRRanBhbHh0YWlJMUdEaXMxWVBEXzAyVmQ2UlJUSWxSVHJGcXBLRUlIRGV4cGtEMjhDSUUwVFBjd0ZPRGFGU3NEcThYbDlyZ2duYzZYZG5idE5EUjRFQWhHQ2hORDZIWHNwOU5Da2EtR3d2SkhKZHBDWUQ3MlEwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>7</v>
+      </c>
+      <c r="G127" s="2" t="n">
+        <v>46014.80902777778</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>GDP report is a much-needed vote of confidence for the economy - Axios</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 17:39:57 GMT</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTFBYRmtwRmNYMmpPdVY4bUJKMzJpSXZtYWJRRUNkU1FjWlJsemlKdFJmeHFmM0hIcjJlS2NQVTI2dFNvTTA3RWFlVUJtYm02Tl84WlZBcEM4N2NtVlkxYlhVMW1BVTc2X1dSNnVKSw?oc=5</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>7</v>
+      </c>
+      <c r="G128" s="2" t="n">
+        <v>46014.73607638889</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Crime Report: December 23, 2025 - Arlington County Government</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:42:20 GMT</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQVGhZM3JpTjFfQUhzMHdOWDZyMkpLNF9NVWhjeVNLSXRzX3FMc3JyLWpycHZRWGtVSFdrWkxENlIwV1lDNlF4QmcwTDY1VXFXd3cybzV0c1J5NnZCaEk4dmlvMWMxTElQSDZNXzloMGltSVB6RTFDSUl1dHZHaDJ5VTJGMndYNkpya2JadmNpcTQ1UnBzM3RYdndXMA?oc=5</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>7</v>
+      </c>
+      <c r="G129" s="2" t="n">
+        <v>46014.65439814814</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>How Did DOGE Disrupt So Much While Saving So Little? - The New York Times</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:27:30 GMT</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNbzB4WVdjVFBJMlREQXVOR3JYampuaFVmbENySG9kMGFTV0dOUU5JVmNhVFptcnc0Z1YwNTkwMy04MHN5Mk5SVEtBTkxJSkFXLUZyd3VJcVFsUDJmcklPQ0VBblNHUnhLTUYzeGVRbHNxeWVveTdtNUxzSnM0OUJJNWJn?oc=5</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>7</v>
+      </c>
+      <c r="G130" s="2" t="n">
+        <v>46015.01909722222</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Current_Affairs</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Consumers Power Strongest U.S. Economic Growth in Two Years - The Wall Street Journal</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:54:00 GMT</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AJBVV95cUxPdFpCNExtbW8wX1g1aGQtcUNfUUZwZGlWM2ExTERyMzR5N0daTEQ2cjN4eWVCX3lQQ1NKZnk3YUptLUhlWlZMOUxGbFZjcDBKTi1TdkJwZG56ckplcW5PZ1dMdHNkR24tUER3eHN0akxSZE1Fc1dBZzR6OUNNTk0tUWdaRmNLZ0pxLVpNLUh5cDRLNFFXcW52TG4xcVpmNWliaHVsbzMxLTFKRXNXaDZqRW9VRFA3TERZdmMtanQ2WmREQ2pjMVlYTURRVXpsbWdUTUhZLXpyYXRTekZueXZtcmFuT2dTeFpDVEdBbWxDX0lJTXhSV1B1VnI5c1lRQi0tLWd2YUFBZWlpaTV2SGtXZ3NXcER2dlRmOTdMWHBtU3hXd0E0VFR1eHRXb0RBN01tTUtTMWNrSlVIUTZDakltOFNEaWV5T0FKWXVKZlBQYXE1RndiWlZyM05zMHgxamw1cFlOOXpiTThRVXQ0?oc=5</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>7</v>
+      </c>
+      <c r="G131" s="2" t="n">
+        <v>46014.82916666667</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Scottish whisky market slides into supply glut amid falling sales and US tariffs - The Guardian</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 18:56:00 GMT</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPcFhaNi1FNk9JekFOc2p0bzhmb2pnb0V2RFAta1pSeVNwQ2RtbWRRdEw1X3JDdGl2SnBaSDlhZVJ5cXhaMFdYU256OGROcU9xU0hyeWRuTmMtZkllQUEyVDBFYUdXSEFuUmZ3OXg3NEU0N2NXblJKcW1fc3FyLXd0OVJ4NmM5Q0Exa1Y4MEp2RkVhemp6WmRCSnhwOWR4UzFqSmdKanZTNXNaY25Qd01UWllQbXE?oc=5</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>7</v>
+      </c>
+      <c r="G132" s="2" t="n">
+        <v>46014.78888888889</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Security Council remains divided over Iran nuclear programme, sanctions stay in place - UN News</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:09:40 GMT</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTFBmMV9NZXNEaE02NWc5cXdac1g5NEtMZGVmMlB3dHkwbTJWanl1OFppWkZpNE8tVmJBM0VSX095ZHg1NTU3WkV0YVdNeEw5dnhzdGw0NlpMMA?oc=5</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>7</v>
+      </c>
+      <c r="G133" s="2" t="n">
+        <v>46014.79837962963</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Port Talbot pollution drops after Tata blast furnaces shut - BBC</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 22:55:59 GMT</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1IQ0t6YWwwT2MzNjFSMExFMzVrcWk0MjFLNGNoTXU4TDcwY21XSmc4ekRxZGEweDgzOXNwcmJsLUF2Q0xpRmdTY1lpQUcwSDNxR0F6VHRJVVg2SjJa0gFiQVVfeXFMTnpzSkR2cTZtTS1JcHBCTkFrNk92TTRJdTRTR3RWT0M3YThiNmhrUVFHcHI2c3JpYlhnUi1iWkRVeU1Db2VJU2lBeXdTU2ZINTJCdGxRLWRmT3MzazFFNlVZZHc?oc=5</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>7</v>
+      </c>
+      <c r="G134" s="2" t="n">
+        <v>46014.95554398148</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>US delays announcement of China chip tariffs until 2027 - Reuters</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 21:17:14 GMT</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPNzVpN1lfdXBzckgxNWVtUVQ5RWFrSmV5UmltVEZmZThPSWFCWWFpYmtORUxBSlN2N0kwOURxcWNfQnJtWWp1S2I1MmFMYmdlTXhudFRydXpaMWtJbDdLa0dILTZUNVVEZ0UtdFpZTzZzWHJ6UDJESmFaTjE4b1AxVGdxaw?oc=5</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>7</v>
+      </c>
+      <c r="G135" s="2" t="n">
+        <v>46014.8869675926</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Navigating Africa’s Container Shipping: Challenges and Prospects - Maritime Fairtrade</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:07:44 GMT</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOVGdGQVptcHZlbVZJQTVaMVN2NEQ1VlBRZ2kydlN3bEo1eWx0THAtQjlsMktDSVVPU3BpZzMybEl2UlNBdW5SVXQxUWtuaHBQYy1ZX2IyWWh2ajBIYklQNnV5cHNxU2V1YUU3ZmdpZ1JqLUVVVE5EbEtZWUpqNVlyZ3VIenNBU1EyNm44aEM4cTZnUVl4Z3R3LQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>7</v>
+      </c>
+      <c r="G136" s="2" t="n">
+        <v>46015.00537037037</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>State Department imposes sanctions on former EU official, disinformation group leaders for ‘censorship’ - CNN</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 23:38:20 GMT</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1qVk5oRkdqOEo0QlFwSmx0SXZUVmktS2ljTGNsbEg2OGltRUo5a2o3SE5mXzZWT2tCMlJNUnpOTk40d08yeDBIMXZrZWlyaFFMc25SZWNLNklSVjUtZ0FYcVFtUm1VVHNHUDdpN09fY2NCQWZ6MHNwT2xrUGY?oc=5</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>7</v>
+      </c>
+      <c r="G137" s="2" t="n">
+        <v>46014.9849537037</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Living, logistics and data centres: the CRE sectors set to shine in 2026 - Green Street News</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 22:06:41 GMT</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOTDgzWFk4Wk9fX1JrY1VKdGJXVnZHSEg1U0hEamRrMUs0SjR2dWp1YkdrMF84SHVza2RSS3NkWE5EaVdfZEg5U2hNeEZac1JiUU5CV1R0S3RJWVpQWXVWc1IwbFJxa1p2Z2Fmdy1UbXI5MGNsS1JqampOYkNMSlJuUF9RVDN4LWtHM25WaFRDVHA3Y190S2pwTVFNSzhaVW1hLXF2M0tqOEVTSE0?oc=5</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>7</v>
+      </c>
+      <c r="G138" s="2" t="n">
+        <v>46014.92130787037</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Linear Faraday instability of a viscous liquid film on a vibrating substrate - Cambridge University Press &amp; Assessment</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 20:45:45 GMT</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxNODc4TWs0SnhzWjJMSVpXNnlYVWF5SWNTMDFWRWdwQ3dFWXNaYnc3enZmaFJsZHdGWGM0WW9UYUFUdEExMWhNemhFSUR3RDEySE1RaWpRX0VqNTdETHBQcWVjUFEyMHpxb0J2a01LcTNqSjhoZkdha280MXl4RmJER1NtNG82bFhReFlZRGNUWnFPTmxRSEdsNXNwWXpwZWtNSllOemV5eUtxejloa005UWMyZlRObGFrS05zd05aUnNGY0xjUHdWTHI1MVBtY0dpNTdrTjhCTjF0azZRUUU3dEpLZFNiczJLeGlGYjZpZUlXQjNaak40UWJqNUE2QndWNktVckRfc09vR21jcnFrdThB?oc=5</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>7</v>
+      </c>
+      <c r="G139" s="2" t="n">
+        <v>46014.86510416667</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Historic Kentucky bourbon distillery goes dark after Canada takes revenge over US tariffs - Daily Mail</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:09:07 GMT</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOdFdwSThhY1ZTdE9ZYTdlbDhCNnROX2hEVnVwX3B4aUptV2ZUSEF2X3RqaXZ2LVloR0ZvYldSZW11M25icVZ4OUktNVVDVjYyZVRkdUVZbUdzUlJ2cGgyZ2c3NmgyXy14dDNuQzZxZ2NSOGg4azMtWmJkaUpyTjZreWF6WUdCOEI4b3F4anl5T21JcF90NVRicjdzd1VFUdIBowFBVV95cUxNSEVua2pRVE9TNnVNanNjZ2RwMThtWGhFbzYzWWdyMV9GTk1aZTVqWUhRX01WR0xSbzdmR3k1UkJfajlVcWZ4SUc2QTh3OTFia0tpaW5sSWNqZjhEY2NsQlVFRHN3aC1uUTZiOGI4VUU0MTlFb1RrZFJ3WGxJeEVYcmFlTm8tMC14ekVjZmN5M0tyS0xHQVJnUFFQMFdaejQ0MG9F?oc=5</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>7</v>
+      </c>
+      <c r="G140" s="2" t="n">
+        <v>46014.79799768519</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Copper price hits record high on concerns over tariffs and shortages - Financial Times</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 11:44:31 GMT</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1qM3pXWURJZlU0eUZ1My10MGJYdU1iMW9iUzNyNWJETFYtUjNsaGNDNUN2MHg0dEIwamRueVlaSXZISVpFR3V4TEVUYldrV0RPS1h4d2R1dlpmWlRvUF9nMlA4YU5OTWRoQjUzUmN1NnQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>7</v>
+      </c>
+      <c r="G141" s="2" t="n">
+        <v>46014.48924768518</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Panama Canal ports deal at risk after China’s Cosco demands majority stake - Financial Times</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:26:32 GMT</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFB1TDZSVWhZcVgxY0NnUE84MERKWnRXeERaVGhlMFJ6dC1takw1UlA3TmNYQ3dqWDY4T0NBWUE2ZHVCRG14WVRBQk5RX3VTQU16SjNITjRtUkZlcXphd3hFZlJDLTQyUk1YTFFRQ1JpalU?oc=5</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>7</v>
+      </c>
+      <c r="G142" s="2" t="n">
+        <v>46014.51842592593</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Trump news at a glance: President claims tariffs behind unexpected growth, but consumer confidence falls - The Guardian</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 01:27:56 GMT</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOQThXc01mRENsSlF3MWlOeVJPcEtReVNFTGV6LWdhUU5kYWpPVnNUWUVJQnJxaDVKZFJISXFRTGY3eV9TdndTUGNfR0d2a0oxTnVnMGhUVmloTmh1UTBDb1NnODE4M0pHend6ZmUxQVVPd0JXRFZ0amh2TGUtNlpwbVY5STUzM2NRTWNKUmVFYUxOam5jd1NqNWNB?oc=5</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>7</v>
+      </c>
+      <c r="G143" s="2" t="n">
+        <v>46015.06106481481</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Beyond compliance: Forging a proactive safety culture for 2026 - Fleet World</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 22:05:36 GMT</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQYXpOdWVLYkN4OG9CdUd4bGxhckZGWEFwWEpQRkliWHM3Vi0zWmVaZ0NpMzRyUkU5azRoN0xPRFZMTEp6dUtObGRwTlRxY0hGNDlPNmZQU2xDbWxvQXdqdlRvM1JUMk9CM2UyLWdGelphYldBaDRXRDl0ZUtBM0pMMWNNaEJKdW9yX2RDak5Fcnc?oc=5</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>7</v>
+      </c>
+      <c r="G144" s="2" t="n">
+        <v>46014.92055555555</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>IIT-M Introduces Groundbreaking MBA in Digital Maritime &amp; Supply Chain - Maritime Fairtrade</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:35:16 GMT</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNZTNncTRxWndMSm1ZWlJvSHlQb0Z1Tzk3U1lwSS0xVUVoSkRGTDBnOHVTemR6QVFkdG5JTkIzZWw1VXRjVDg0clBxMXNCbXc0V2hfMEN0NllLQUZzWVB1OHJNSFlFMjBNdGdYblgyRUxsVXA5dGkxa2xWNWx6cV8zRHJNOExybXYwa0tsWVlvZV82aW8xaG5zYU0yRU5hMVlk?oc=5</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>7</v>
+      </c>
+      <c r="G145" s="2" t="n">
+        <v>46015.02449074074</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>China to Develop New Port in Kuwait for Regional and Global Trade - The Maritime Executive</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 23:21:06 GMT</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMDBiQ1k2clhYNTVpRm1xbTZmRlhMV1ZqdGxKdVo1eDM0T0VfWW9KUjR4Tkd6X3ZWZy02emNNa2Rkd1RiMlBNUjcwcHp4QjlFbVBDNklpYWltd3A3dEx0T0ctWXU3cC1meVRxVjZnWkdiZ0Z3dFA3eGVpNXh4N3JZVWFaS3lQOUJidGEteEhnYXpnNW9BdnRna2tKNHVCVUQtQTRsQTJCcw?oc=5</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>7</v>
+      </c>
+      <c r="G146" s="2" t="n">
+        <v>46014.97298611111</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Man arrested after €3.7m cocaine seizure at Rosslare port - BBC</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:07:11 GMT</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBzNHRQaHZILXNKMl96OUp0NlNZVmtKbUNEUUYyS2E4LUpBRmtpSGdXbjROdG9qV2ZKeTA2VGxucURaUmt5NW9hU0J3NGh1RVpQcWlqTWtjeFJGd9IBX0FVX3lxTE9PV1BXd2VJeENoZGR0eVBVZ3F0UmktU3V2dUxKTGJDQWwxN3Rld0RBY0Rib0pydzBRUUlOb09PbloySlluQmpWN09PRTI1Y0RxdVlhdFlnRzZXV283ZjZJ?oc=5</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>7</v>
+      </c>
+      <c r="G147" s="2" t="n">
+        <v>46014.50498842593</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>AI, Tariffs Fuel Big Tech Layoffs - Global Finance Magazine</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 21:33:06 GMT</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE1HTHJJZFNOVlRod2t3OVNkWjQ0MXdfWmVRU3ZrYXh0OWY4T0FSd0VydG1JLUZJcWYtcmY0NkRfazFZZEh6dWtKNU9WaXJhdFl1VWV4dzQ2SjdqdHJBcHVNV2RrTVpGTnc?oc=5</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>7</v>
+      </c>
+      <c r="G148" s="2" t="n">
+        <v>46014.89798611111</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Strengthening supply chain security: Preparing for the next malware campaign - The GitHub Blog</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:01:15 GMT</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQb1NNOW03OWs4N29yNEhnR3YtTzY3Y0pac1BIcjY1T0FJRmdUNVJ5Uk1hWkFjeTlYdTFTYUlRUmFjeEdpR3hiQ0E2WkFqTGM2Y1FnMVU3allYSUhpQ2J2ZUZKTzloeVpnMUxxYVgyRTZNUWFpQVdING1rMWV1c0xPVG1VaW10cnhQd3NiT1NsbzNMX1NPRnN1NjJyQURQNDRRbUNlQ0dWbWZWeTVMMU1nV2FpMmx3OVpVbktOSk8yRzZnRXFGdVE?oc=5</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>7</v>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>46015.00086805555</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>How brands shifted marketing and media strategies through year of tariffs - Digiday</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 05:02:38 GMT</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQUW5JMlVDbUk1ZFpTWTM5S19Rd1piMXgxRk1RT0twZVk1Nk5LZ1NNVEN1QXd0NmpxMlZSVFZhT0pDZ2xrOEhLTHhtdElycXBJeWxXMnZOaERGMGFqNXVXZGRzTER6dnNYZzR4WmJNb0E3WWJIeVB5UExVMFVMaVhsVUx4RGdGX21UVVVlRmxDaHVSb0dTdUk5eFgybkZPVUxOUDlCNUM0NA?oc=5</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>7</v>
+      </c>
+      <c r="G150" s="2" t="n">
+        <v>46014.21016203704</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Shipping Giants and Insurers Unite to Combat Corruption through MACN - Maritime Fairtrade</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:29:54 GMT</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNRWU0dkEtSnVKU3dWTDZTcHdxUzdoTHFjelE1UFdPNktRRXVZSV8wbVhydldHTFZLLTN6aUphZ0lTXzhVcV9qajJUX2tXSnkxdU96dkVrZmhMd2RRSkVUVjc1b1ZzckN0R19IaTV0bko4aEZVRUxBd3QyRzRXWU1RMWRUaFdiOTBQT2lQWF94LUdhMWxzUm9DRGpjaEY4RmhO?oc=5</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>7</v>
+      </c>
+      <c r="G151" s="2" t="n">
+        <v>46015.02076388889</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Huddersfield Town press conference: Lee Grant and Bojan Radulovic ahead of Port Vale clash - We Are Terriers</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 11:53:59 GMT</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPWWtKQ2pEX1FtemM0NHNlQ2lQNVJQczZzTUtjYVl4RHhyRGlxb2UwODhtRW1ld2dJLW8tTG5xQzNlYWpzMU1HQzV5YkJCeEdXbnpIUnliLVV3QjI3R0ozWjlpWFJ2OElBY0dpRVVKSG5sM2RNdU5ZQnV5WjRBUWdISTY2eml4ZmJlNWRHTFhlbzA4NEh5Y2xkM3RQX1NNT3dYd0VYbQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>7</v>
+      </c>
+      <c r="G152" s="2" t="n">
+        <v>46014.49582175926</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Malicious AI Models: Risks Across the AI Supply Chain - wiz.io</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 21:18:36 GMT</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE5lSkEyeHlCMURVQS1EOVJ3Nm53Sm1SMUpqSl9OV3dRdm5aSjVFNzNvYndrTmZoanlWdFo4UXd2OFFfQkdGZmZfNkRjbDNXTndTUXZsRHB1a0o0N2FDZHJFUmNiMUktZWItYkE?oc=5</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>7</v>
+      </c>
+      <c r="G153" s="2" t="n">
+        <v>46014.88791666667</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Pacific Basin Shipping orders its first bulkers in China in over a decade - Tradewinds News</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:55:25 GMT</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNdGlBRm8tNVBJUFMybzhCYUNGclFYWHN0QmQ3c0tPbW5zd1RrZ3lFU3MxbGlwODdQQ2JmeXY1bXNyS1dyLWphY2phTTRWVC1FMkgtTzBLUEZCT0JLQklBWlh4eXhRR05VTHhkaWtFTmo0S3BBWEZ0eXNxc0MzeUV0b3JjTnh4cTBLY0d4ZVRDRm81UFd6Yk4zU2twUUdibHB5S00zcEl5eC1QU1A0dENlYlpjbHpzRE56U0xJNDZ1NTVsUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>7</v>
+      </c>
+      <c r="G154" s="2" t="n">
+        <v>46014.5384837963</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Sumec Marine Inks Contract with Shanghai Jinjiang Shipping for Two 1,100-TEU Container Vessels - imarinenews.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 01:36:04 GMT</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFB2MlpLdHVUY3RsbHpPVDNwcE9kT0RrRVJUZ2RSdHAtRjF0ZVF2WHlmSlplWURkVXhEMTZTRXRmbVdrVV9hem5nMzBNaFVnTlk?oc=5</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>7</v>
+      </c>
+      <c r="G155" s="2" t="n">
+        <v>46015.06671296297</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Might We See a Streamlining of EU Digital Compliance? - JD Supra</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 22:33:36 GMT</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPdWVlWEtyeGYwOHNHVXk1UVFrd3p3dTBGY1JxM1NLNTZIaWNqOUpwR3pYVlZpU3RncGhlSWtJdUtOT3BYeUl5ejRhQTIxSG9qWTFHbGxYRHpNN1lHVFN0SW5RRFJQb3JfVHdhYnJlbC1sSHUtbzFHSS1SenFMbmtNcEh3?oc=5</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>7</v>
+      </c>
+      <c r="G156" s="2" t="n">
+        <v>46014.94</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Russia Risks Logistics Crisis With Winter Troop Surge In Ukraine - Forbes</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 11:40:03 GMT</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOei1hdFFrTV84d2UtYXlaMTN3Y1ZrdjJlV05GajViVmFwWTg3TFhtS2VVNTVidXpLOW5ZNFdoZ3VocnZTcWpsY2t3WDYzSGcwV296bVdOTG1HeUU4ZVZTVG1fd0t0NEtGLW1ySlpITnk2ZWllTkZRS0FtWHI4SDU3bGJ1dmtPNzhVWU9QWUlHTUdjUFR1Zk5KUF8zWDEtd1lMZU1QS3cxcmlfNW93ZkdNaXB5Nkd0VllBa0E?oc=5</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>7</v>
+      </c>
+      <c r="G157" s="2" t="n">
+        <v>46014.48614583333</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Peter G's busy Christmas: United Overseas snaps up dry bulk arm of Norvic Shipping - Tradewinds News</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 18:35:45 GMT</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPSUVMdXk2UmpCMGNfbG04M1J0eU5COGJ4ZzR6RjhweDRuRDZTOTVqRzBJc1Z2THFyWnBDSU1yUE90T1Zjdkt3djBLOHFfREdSaFRxTW41RV9CYmg1UVRLWTVFVDNmRlpjUzZwQ2FDWFM4OTY1MDBIekExNEJBaTBUbE5GWlk5VmNIbW9OUXcyMTl6TUN0VFIxUkdpeGd1bGQ4RjNsa3RUZjhraEhHV0xycHBUbE1zRGRPWkw0NjBBLWVNREQtVzJ2Uk1BQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>7</v>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>46014.77482638889</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>UN Reaches Shipping Emissions Agreement Amid US Opposition - Maritime Fairtrade</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:34:56 GMT</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQc1l4ZzVWUnFGOFlMSC03N3BnTDBIWldpZmRXRVNxSHVfM1ZUNmZxTW12NEVodWsxYl9XVHFmMlB5REZlcWtHVkp3bktmSnBWUWJYaU1zdkZKQnpVQjRlZlN5THhPa0I5YXcyaFRLTGdZTWRjVXhwMFU5dXZMOXhRUWdUVFpnUk5CU2pHVXdoRWk4LTg?oc=5</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>7</v>
+      </c>
+      <c r="G159" s="2" t="n">
+        <v>46015.02425925926</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>JINGDONG Property Announces Acquisition of Grade-A Logistics Asset in Leicester, the UK's Logistics Golden Triangle - JD Corporate Blog</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Mon, 22 Dec 2025 11:15:24 GMT</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQT3M4S1p0eEc5WEIxYWdFa0RGX1F1Q3hVcF9NUFdKQXFadFpfYUYyeGpTY2RUSVU0QVlHREU2azFrbWZ0T2MwaUZLUVFpM0Flc2VLNjZwZmNobDc1LVdRNHFUZlE0UGlJWlFpSUlNaHRWYlBGb3pnOFhoc2hvXzY0U2xoaXVNaTNBSGhqYWlTMFJEenFZTWpMa2ZnMU1VWUk1dWl2RnBjWXFtRFpnUzQ3a2drVWprclFndXdHVlBwbVYyNlpvZnQwdUlaN201MG1KTy1GVDNaT3VqQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>7</v>
+      </c>
+      <c r="G160" s="2" t="n">
+        <v>46013.46902777778</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Supply_Chain</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Dry Bulk Shipping: Global Iron Ore Volumes Post Slight Increase, Despite China’s Imports Decrease - Hellenic Shipping News</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 22:05:31 GMT</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOWFdIRXpWX3l0Q2UtSUNtQ2ZKdUdEdmpzS2xxbVl2Yk1Pd0RpMzZxU1VIcVFHdU90YVJHbmoyeGFQUDJRem1lMklOaGtfSHJLeWxaNFdkTXhSRG5NaG5yYjBoM3NacWZPakFvczJFS0xCRjZqVVdaSldOb3g3bVdGYVV3eVh3b2owcmExUU9jTFhBbjRfMk1KeFlGU3preTJXWU5FeHZBblJMV1Y2dEdubDdMalBiRl9jNFBwUHhxMFhoRzgtYTAtQzRBTmQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>7</v>
+      </c>
+      <c r="G161" s="2" t="n">
+        <v>46014.92049768518</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>British police detain Greta Thunberg at pro-Palestinian protest in London - Al Jazeera</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 14:12:17 GMT</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPTUhjNXV4a3ZmajU1N1p4ZXRRNlZYdDR6S29OZDRCTE5GSWNrOV9uT2RXNUwtOUlMLVZkVUYwaWZOUjQtMlRka2phTUQ0aGJ0UDBZSWN6UWk2aV81RU50OEVzUHVvcmwxYWVFX2k4R2xLNUVuZlVKQkVFWk40VlhxZEVtY1d3cWxfUHY3ZkZONEdyOUt5ckZsVkViVkVtemxQeVE4SG5uSDNmNm440gGyAUFVX3lxTE9rRnVkLVVIajB5WDNqN0JYcmN2amxiMDFYMkdOZDhvWlFyN2lrUS1HRUMtaXdZdGI2MEpkX1ZhOWotMGpMbmoyLUpZOEx1XzItaTE4R1FBOWRhZWF0U0dOWjF1VHR2c2twQ1JxT3MxemNHRUtPQkFUWjZDQkppR3VORmxYMHdlQkk3Vnl1c0pxRnB1WFNDMlVLUjc3dHl0aTU4Zy1zSEpIOFdyS3c1Rmw3SWc?oc=5</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>7</v>
+      </c>
+      <c r="G162" s="2" t="n">
+        <v>46014.59186342593</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Amova Asset Management strikes deal for Malaysia’s AHAM Capital - Pensions &amp; Investments</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 20:45:00 GMT</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE9BUnJzSk5pSjBzMFJuMFptUFNHcURYN1J5ckszVE5hV01Fc2FOSG1fc0NoSzJzU0N1cU1naERvc2p4Z0xSYTVsaVFBUERNTkNoSm1ORHFDZl9aRnl6TmV0SVhkbmQ5V24yMDRDczhDQm50Qk1yTjB1Xw?oc=5</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>7</v>
+      </c>
+      <c r="G163" s="2" t="n">
+        <v>46014.86458333334</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Massive protest outside Bangladesh High Commission in Delhi; protestors clash with police, detained - Asia News Network</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:36:38 GMT</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPRmd3T0ZBRGhFakNJa0tzcVJ6ZmstRmF3QzVjQWp4ajhkOW5COS1XTk1FZVJCV0hyV3JUWmFNRjlFRFczRGJCRFJ1a3h6bmxDUVZRTFFxTmcwemp3bGRyOTJ2SmRwVjd5eW9SY2RtY1F0ekdYSnczcGxleUNCQklTUjdVVGhqbzFLRTJOQmh1UzNZcEQ2NWtOUmRVZlpfLWZZN0c0eFlwU3pkVExtNzZJZExyYjNnN2J1QVpxdVBRa1c?oc=5</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>7</v>
+      </c>
+      <c r="G164" s="2" t="n">
+        <v>46015.02543981482</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Protests over fuel subsidy cut leave police injured in Bolivia - upi.com</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 20:07:36 GMT</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOS0VsMWpIemtWY2M2RGZIV0FXZkNTNG5CN3JQT3psWDJxejQ2c0NkR2x6d1FveUpUNHIwMzcxaGpqdk1ZcFpzeVZpWnNTcUNfMEZWMW5DbENZbGpQSGNBTklTOHIzQXN5MnZubTNhbTlpVlpjV1lhMzF4T2l0NVM3ZHhqaXNzaUc4OG53V3BTSkRLQ2Rzd2VMOW90QWw2cXNrbnNZZV930gGrAUFVX3lxTE55dzJ2QUc1TWpnWUlFcHNYYlZXaFZlVC1JaUZaZUhiSGFQZXdFVGxtMEFxMC1IeVdMQzN2X0lySzg0UFM2MzZxNzNoX1RVdTRXRWVCLVpVSFpSNWlBZ0pwQkZ0ODFucHpDRGJfbzlMR1JQTklqRUZYYjQ3cUtCc3lNa0dxcG9pN0VqbFMxcUpIdTR2bEwyWXE5andiSjRNMFM3R3BjUnNmZkczNA?oc=5</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>7</v>
+      </c>
+      <c r="G165" s="2" t="n">
+        <v>46014.83861111111</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Minns defends new guns and protest laws after marathon debate - Capital Brief</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 01:01:00 GMT</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQWXFlOU91YVZpRUFyakxOdS1WZDlyQlo0ei1FQkMyRFd3RnY2MGVwV2JPUjdiYTZVbE9jZV9nb0FYeGV3bWpaN0xKVzVSZm9abHhyV21GVXl4MnRsTDdqMmJfTHljSktqV3dNZDd3aEhMZlp0ODNXdXE4Ykx5WndjSXA4YUNZUmFQbmFGMHdGeTRWbmJEVEdYeDhKaE12ZHB5aUFQY2VLNi12OTl2YTRmU1FmTzVoc3hRZW1STnlram5sZEVnOGQycHJyMl9nRG5HaXNj?oc=5</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>7</v>
+      </c>
+      <c r="G166" s="2" t="n">
+        <v>46015.04236111111</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>24 Wounded in East Jerusalem Amid Police, IDF Raid, Red Crescent Says - Haaretz</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 23:08:00 GMT</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwJBVV95cUxNOEU0WVNTSF9kNWU4dVp6U0RUYmwtT0NNeVlobDBGenVfSDdTU2hGMExJekM2YXgxYnpUWWR4N0VjRXM1ek5fcExwcnpuamppRGpuMUVKNzU0M2Z3OEY1ZXVXLV85S20wWnhuWmFJbDdzVkpNMndleE1FbFljSEtyZXlKUk9RSUt3TjlFNXNvQWpfZXllb1ZjUF8tR3ZualJROEo0bWVLN0xUdkQ2QkhLZjZzaVlUS0JYLWU5ZzdVV1d1WkQzQnpScGw0SVI1WF9wSG1SMlV6NE5UcGF4WWZRbzdlSWNUczZlQkJIZG1QSFI5LVd6QXdIb25rVVV0SEZMTzRocGYtTWxXRzV1bUxxRHYxMWx6VGc?oc=5</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>7</v>
+      </c>
+      <c r="G167" s="2" t="n">
+        <v>46014.96388888889</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Ainslie strikes Oakley Capital deal to fund British America's Cup bid - The Straits Times</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 07:13:00 GMT</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPZVVsQ3BoaEgta19weWl1ZVlvUjlmUUl4RF9WWHJrRmNUcm9hc3JzUWY3bExMd0hmM2UxWFNVcVVOOUphSkNmVjcwOXJSUXg0N3dTTkJkR0t2OXZ2SF9TdlYySWRHSEMzRi1MSVcwRzVjZnJXOTVtS2oxYjl5NUc5WFdsSDZGR2IwNVQxQ0xYVDQ5MWhnbFFnUUo5cWlhMjFtZGhKeVNn?oc=5</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>7</v>
+      </c>
+      <c r="G168" s="2" t="n">
+        <v>46014.30069444444</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Reps approve Tinubu’s request to extend 2025 capital budget to March 2026 - Premium Times Nigeria</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 17:04:02 GMT</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNajdFakpnYV9XZ2pCdHBZblJwd2hmb21TekNYaXE3Wk55Wm9MdThpU2VmY19oUTBzbEtCNkwwWlAzN3V1cWdlbVdCQTItRUxCcjNZbE81aWJ3ZG5UMEFic1BqX3NpVGxldUp6dTR0WkhMclM3a0wtcEF1MUg0dzg4a3c5c2lNT3pFWmdxLVp1RmNxdlNmMUZPSHkxYVZ1RW5SdE5XNHl0dE9ZbVg0MjF5amJaazdINjI2aDN2d2ZzWnViRDFNaGpHVg?oc=5</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>7</v>
+      </c>
+      <c r="G169" s="2" t="n">
+        <v>46014.71113425926</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Protest</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Bondi Beach attack: Father-son duo planned terror strike, say police - newskarnataka.com</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 02:07:14 GMT</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOTkNRcnRZTFJwaHNjNi0teXBfZVRmQTljYTY5cEF5WWY3eHE2cTBFYUdkY0pVZlVHSE9Tanh1UWdTM25GU3ljd1FmMHNBdGRPVnJBcUxHVmVrOEtYOUlSblkxQzBDR3ZOZmRlS09tOGRyWWJrdWdXdnpJR1hZM3YtVUVmdFZxZGMycXZJSU5GR2F1WEQ1bm5JLTN2aDhmV1I2eHhvZGpscXIwb00?oc=5</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>7</v>
+      </c>
+      <c r="G170" s="2" t="n">
+        <v>46015.08835648148</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Elon Musk, AI and the antichrist: the biggest tech stories of 2025 - The Guardian</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:22:00 GMT</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOTnhaUURYZ2laU3hMYXl6a3Y0N2pXSm80UGs4dmEzVVd2RzJVWnBoRkhvdnUxUjZTMWpSemE2R2R0M0pvMGNLOVJDOXFBUUpkWjZDdWtKdURBMHplbndSQ3E1LVREdXYyMGRkdV9WSVFFbE02OVVBWjZNd3pxdXN4VFF3?oc=5</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>7</v>
+      </c>
+      <c r="G171" s="2" t="n">
+        <v>46014.80694444444</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>AI and digital tools can empower civil engineers, not replace them - New Civil Engineer</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:25:43 GMT</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNbGM5SEVHUUdFaWxqVEc2bi1fZW55ZkxxUVJmRzExRzhlMzZkbzV0VTFIWUZ5Y0h1MmExRVdZVWZEUVNiYjRlbkttWFRxSElzUkdWU0dLMlp3RFBidm0yRTNHakV2cEtQcWlNdjRvdEhEUDQ4VF9McHA5TWdvQUZMMGZnbjNmZS11UWNIN2JqeGZhZWNoRmI1ekVMMG90cjByVUxkNXljM2lsSlpRYXI0dm54VTFrWEJsR2c?oc=5</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>7</v>
+      </c>
+      <c r="G172" s="2" t="n">
+        <v>46014.51785879629</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>AI View: December 2025 - Simmons &amp; Simmons</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 16:18:45 GMT</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPZWxsa3JwX25DZm9tMDFmWkMxcUhqT3V2a19JcTY5QzJwQi1ZTkI4SUFMQ1RvT0ZVM1cxSWlHdGhlVG4wTG5vVkJxamlPNVdpbmdOVTZFMWlyWkc4RTVpb0JLZGZlT0Y4T1RxMFA0MENJbjR2WVVXZlptOUlLd1gwenlNVk40VDg3cVVWLVg3aERvSDBlUnU0eDZNZw?oc=5</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>7</v>
+      </c>
+      <c r="G173" s="2" t="n">
+        <v>46014.6796875</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Hyundai Motor Group Strengthens Software and IT Leadership with Key Executive Appointments - hyundai.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 01:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9ON3RCNjdNYXJFRUllM2trVzB0SmsxaW8zVy1BeTNxZE9mOGR2ekxTNXRMRTZZSzBVYlBveWpSSV9RWnlIQnl6aUNJaTM2TXM3dFlBQ1NldGlUdmJmZlRqZVViSXdNYm51M1F1QlhJUVM?oc=5</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>7</v>
+      </c>
+      <c r="G174" s="2" t="n">
+        <v>46015.04166666666</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Dreamlines-Cruise1st targets ‘significant growth’ by developing AI and packages - Travel Weekly - Home</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 08:55:00 GMT</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOb0loVVprNFBHUmFlQ0h6cUhTSWhBcmNfQ2xKUzZDZWZ3ajQxbG14X25GVmVYa3c4dEVNcmhXT09JU0lhY0ZBczFfcjdacWlySENMNWFVVEFoLVBnZDRLaTNidlpmR1R6aS1Vd0I2cU42UUxiWG15Y3RuTmE3WHNSN2tQUjdDd0JJZEU5Wk50VjBuZk9jT2hyUm9xalZRVGVwemVwRFBlNzB2RzdxR1RFLW9iT2FtUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>7</v>
+      </c>
+      <c r="G175" s="2" t="n">
+        <v>46014.37152777778</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Researchers use robotics to find potential new antibiotic among hundreds of metal complexes - University of York</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 14:35:34 GMT</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRUNqWnVkWVZrOWh5NGtTTHlZa19ubzRwNFB4eFF6TElmRFFBUFJZeWo5UW15N2tMNXRlUkdPOHV4Vkt6dVBQSWxqMlZvcnVBLXkwWUpfSERBZ2tPdXp4RmlKN0YxSHRvTXVvSlFrczA4NVdUZkIyUlc2WG91OFd5RnZSNjR6UUpxVTNwS1ZEdTR3d1E?oc=5</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>7</v>
+      </c>
+      <c r="G176" s="2" t="n">
+        <v>46014.60803240741</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>What Is AI Threat Intelligence? Real Risks to AI Systems Explained - wiz.io</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:32:27 GMT</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE1NcjZmWFF1YXhxaWhvMnFUbDFVWmRYdVdXeEdSZnp0SXgyZndNMVk4VzJxc2pNNG9PQlY4TGQ4UllFcHRxZlJnd2YxMDNnek1rako4dFJzUTFnZUd2U25YRHlYUmF5TUoxVWpvcmpzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>7</v>
+      </c>
+      <c r="G177" s="2" t="n">
+        <v>46014.81420138889</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>2025 Cybersecurity and AI Year in Review - Holland &amp; Knight</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:13:21 GMT</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQN2Q3SWc1X20xVUd6eHUwdkYwWFZ6MEhMdlhFZTVrUEU5Z3pBUTQ5alhheS1LbFZ5SFF2RGM5RWIxTEprb1ZSaXpfQjlKbFdOLWg0c0ZGZHBGTnk0U2JvYlg2b29Xd1JFbkxTbmxVUXJFSHpEZUtLeG9lODNiVEh4R1Z0aFAxcF8wMVIwNHItYll6VVFJbzkyOGNjTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>7</v>
+      </c>
+      <c r="G178" s="2" t="n">
+        <v>46014.63427083333</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>CISA Releases Cybersecurity Performance Goals 2.0 for Critical Infrastructure - Inside Privacy</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:17:07 GMT</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPSmFjNEJUaHRwRUlMOTU0Mm51UXhpX0hIQkNkdkFHX1hLTWpYTThLdDl5cUh0SldBOXllZnk4dGYyYXFlaHE2UzdxanZtQXVlZzZlMFlLVVladTlLcWFKYWZvUlM4aHY5MnRzOGpvMjNiTlM0WWMtZnZtRllISUJSdVZRZ2pTMUhDZ3N2QVNGVklsUU1ybldSN3JzdHRYd2Q1TnptVjQ0S2RUWkVRNmpTT2M1NTNYN1hpajEzbTFLbw?oc=5</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>7</v>
+      </c>
+      <c r="G179" s="2" t="n">
+        <v>46014.51188657407</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>The Convergence of AI and Cryptocurrency: From Digital Transactions to Agentic Payments - Chainalysis</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:02:37 GMT</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE5aVm1uTFZCY0kxdjFLVDRiV0ZKSFBYM3BKdHNMdm5UNDhIeTUwRUhIbVR4R0VvZ2JEQUZuODRZYzRrcEpQYXZFdUQ3YmtEb2VUNGVPS1ZaWlBPblB2TzBoNHAyOEYwYk9uZDlWSnNUdTcyQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>7</v>
+      </c>
+      <c r="G180" s="2" t="n">
+        <v>46014.50181712963</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>NIST and MITRE partner to test AI defense technology for critical infrastructure - Cybersecurity Dive</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 19:50:46 GMT</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQMEVNTmF5OUlKQlZFX3VkWWxzcG5qOTE3LXRSNmpVU0I0SDJrRThNQngzUDdrdzZuSVpJOUJ3dGhNdmF0OW51Z1ZfWnZOZklXQjVNNWNNTkZ0MjU1QmpiMkpjRzZBMngyYVVZQnM0NGFJekJNcjZKOFhYZkZrVkZTajltbVZvdERMUnIzZWdjRWstMkUzXy1YZEhrUG83djNOVVE?oc=5</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>7</v>
+      </c>
+      <c r="G181" s="2" t="n">
+        <v>46014.8269212963</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>The top technology trends to expect in 2026 - National Technology News</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 09:32:52 GMT</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1MdmhrUzNpT3NZOUd3bzVhY2ZHOGo2QWFNV2pSSmJhWWd4bUtXY3FjWmZ0YUtVX3EzWmFuMFhYNjExQXlCYlhxV1BVVE9pU1d1dVpERFkxX0ZOTFpDT1lOaU9jOVE3dm1QUWxfS2JqaHNyQllheGZBbDhpZFM?oc=5</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>7</v>
+      </c>
+      <c r="G182" s="2" t="n">
+        <v>46014.39782407408</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Motive appoints AI innovator to board of directors - Fleet World</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:05:23 GMT</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNTXZoemZGWFZoTU9PYlp6eTFjZWJ2NkNTQmZaMnA2OGlidjhKSGFkam92NVJRV1FMUGpNcmRZS2daR2ZlUEhCSVpROUMwVW9ORFhJZGNnRm5qZGRBb25EZW83NUEyNTBzVmdnZU9VV0g0REthaG94azFHRzAzMWZGbU9n?oc=5</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>7</v>
+      </c>
+      <c r="G183" s="2" t="n">
+        <v>46015.00373842593</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>NHS boss warns against asking AI tools like ChatGPT for mental health advice - The Mirror</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 00:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNX3BpVGF1ZmVQWDI3Z25haTlyRzBVQXU2bGpNYzZkVXduWEV4T2pRVDlKOEI1YTJxaF9ETnJIZy02RGlnS3A1MDBWRzBmdmpvd0lqQldTMlRIbld5Q1BwWVN2anl5NHFaVEdFLURSUTR6bDhuMS15UjZFVG1KTGMwNdIBhgFBVV95cUxOWHRUMnNjSG1kZDZlcVJTN2M1SE5hX015R3ctSVpHVmdMTGp6V2h0WDM2bEpzRWUzcVZfUWZUWDVmalRyMjM4V0gyQWZjSDBoVFBxMEtMdnpDa2xtNU5saFNxakVPZEduUzZhSWNZMEdid053bEUwSUJnVEZpYzVaUVdXbFBFQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>7</v>
+      </c>
+      <c r="G184" s="2" t="n">
+        <v>46015</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>RPS appoints director of finance and technology - thepharmacist.co.uk</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 10:28:05 GMT</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQdGdQS29RTm9HZUNpeUZZUnMwRFY2MEh1SnlJR29xN0xQM3ZGQ3lqMjFjREQxRW5WYXhkTUp5ekdKbng2WUtmZVNvN3VEZWRhUGE1ZmhWWFZneE9TYTVFUEZNWGxJWUVqOTc2MlV4M0JYOTdEbnhnQ0RBUFhYU3E2ZXp6M0c5bW91c1EzS1Z3?oc=5</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>7</v>
+      </c>
+      <c r="G185" s="2" t="n">
+        <v>46014.43616898148</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>2025/26 Reflections &amp; Predictions: Paul Greenwood, Clifford Chance – AI adoption is at 90% - Legal IT Insider</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 13:20:31 GMT</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQZ3ZlMkRWQkJYSEt6WlZyMWFXQ3pLQUd6UkRuTldVVTd6ODgxYzVjQlFGdWd3QXdOSlR1M3ZJM1FTWUo5TzdZSGdVUWJTRmtIaVNsbTRSNnVidXZONDVfTmYybk9HaGNzTTg0eUdzS0JvYTFURDVndDZmWGh4bkJiOWpISHU5OUZYMFBaZFpOc0piY0t0M0JZa1JVNEZUQVBPd212R2JfWXJCYk5uTlF3clY0d216ZmREYW5zaG1lSGk?oc=5</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>7</v>
+      </c>
+      <c r="G186" s="2" t="n">
+        <v>46014.55591435185</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>What is California’s AI safety law? - Brookings</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:10:57 GMT</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBrWnM1OXlQRFRkYWQ3c013RkhGTlR0ZjY0UXJOTVgzVUVOOC1aS2VEQndxQi02X0NNOURTOFlUNzBVeHpqeGZWM2k5Qm9pS2N4WE1haUtaZWdYQkc2M3pONWFRdXlEbHVmdEJEOS1fOFAxOFkwT1ZSbA?oc=5</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>7</v>
+      </c>
+      <c r="G187" s="2" t="n">
+        <v>46014.63260416667</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Why most AI adoption strategies are failing and how Wrike's research reveals the path forward - The Manufacturer</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 11:45:35 GMT</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNRm5rc3FZLTZiQTdKYkFpY3BYdEg3bWtXdHdHYzFTcXUtVU9UMUcyeUZEWFM2UDhidGZwczJvc1dJc3pSTVNVcTBHM2ZjZ3FMUHBvY1ExOWQ0a05JZ0tVMG5ZeXUxQ2w1SGxrQWxMX3ZaTlBJNjBsQ1dTZTZQQ1M2dlJnVTU1eG9GNzk3V0VOeUV4SmJ0Uk5nRWdOemt0dlNNS0o4bWhSVGYzcVZBWVRlUG5IeFRwb0MtNzJSLW9ub2FhY0xRNC1ETktwbnhPLXc?oc=5</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>7</v>
+      </c>
+      <c r="G188" s="2" t="n">
+        <v>46014.48998842593</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Cybersecurity Predictions 2026: Preparing for an era of relentless and intelligent cyberthreats - Intelligent CISO</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 13:34:46 GMT</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxONFVuRHFMQWE1ZHRYYkhfMjRvTElKWmc2dzREUkJLWTFBeVlaNndHSTA3TDRZTVlLcnhxdzdSQ2xwLTJsZU5BcjQ2X2RXUUNRbUJjTk94ZmVBSm5VcFZwNFBaaUhCc1gwRzJWV1dldHNEcUNpRU5SejBEeF92TUZMYk10XzltSEhQX3ppZDNDeTBLczNyNkYwUElvYnA5QktaN0szSlJvcFB1S1BvMDNxbzA1X19zakFreW1ub0VUM2pxNVdMNnQ0WGl4NmhneUFWcWNlUA?oc=5</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>7</v>
+      </c>
+      <c r="G189" s="2" t="n">
+        <v>46014.56581018519</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>How can Canada become a global AI powerhouse? By investing in mathematics - The Conversation</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 14:06:08 GMT</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNYTRoTWEwMGdpZVd4azhwT2dhd0ctNHRPSWs4V3VoZU1BSzRwTEZ2QWhyWW04b0Job1REbVdXcXFzenZ6d3VTZHE2YUNhX242dlN3RmYtUDhaRHVrcTE1eW1ZYjYwTnFBdWRMZG50eXU1VE1INUJ5RU9WSl9uTjktVFNVM0Q0Y1IzWkVjQXIxdURabW93ajV0dDB5bTRjU3FaTkFiUWhHNEpNU0E?oc=5</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>7</v>
+      </c>
+      <c r="G190" s="2" t="n">
+        <v>46014.58759259259</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>How Automation and AI are powering the Gulf’s digital future - Intelligent CIO</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 14:47:54 GMT</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNX3IxMGJsWVhtX2c3QkhOYmt0WG9jOUlkSEhOcHhubzhXY0QwUEZJdDVZdjBpNmlGOXJ1X1ZwSzBUSFhodHJiOGtPS3RISzNVQXpWcWtNdERIOG9tNXZZSi1hSV9lRE43bHpwNWVCcmxRQWNINDFvYWJIY2FHclVCLXBZQi1uRkpIa29TU1lKZG9wajAwckFGcVFrS1RuUzNWOGV3R21XbjY?oc=5</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>7</v>
+      </c>
+      <c r="G191" s="2" t="n">
+        <v>46014.61659722222</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Kamlesh Jobanputra Joins Edelweiss Life Insurance as Chief Technology and Data Officer - CDO Magazine</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 13:30:00 GMT</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOU2ZmZG1odUxobGY4ZURqY0JiV1llR00wY081akNTZTEyR080aXd1UEZKTDBUSkZHQkNkdTRuYWVFVWNOYkZYZm0tcW01WVN5YWh0T19uOGRIclUtTVhuRHZnSmRlOTNZV3A5NmlXci1XYk5pd3huOUlGb1ZuNmxJZG9sWkwxM21OSlFzVzhWZmdITEJPM3BlVkVfTTlkbjFiQWJoWU9Zd2dFV0tlcnRGTlJydjVfcE9sbnlVWTVGVlNUTzVta0QwWWZtQzc?oc=5</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>7</v>
+      </c>
+      <c r="G192" s="2" t="n">
+        <v>46014.5625</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>The Continuing Expansion of Algorithmic Software Laws – Best Practices for Companies in an Evolving Landscape - Winston &amp; Strawn</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 21:45:00 GMT</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxOYURtZTBiNllCVTdnZ3Q5ME9IMVppNE5hUXJPcFJWdFo1SjlVZElObHBOeWZ0Q2lic2lSSlNMSlNwQ0wtTVlxTE1wMVNlMjlIRmZNS2hSSmRjczRYdVhVci1JaUd6Sm9zTnVTdW5XTjlOYU0tMUpkVW9VTE1qRHJWUGlJdDBkWkpibTQ2bHY5RmFRZVliNk54U18xdWlRSVdmUFVCc2FvOHV2TE9YMFJuOU5WaW5vN3Fma2h2MWZ6MFlnVUwzQVk1SVBiM2tOOUtYOGVITDg2S000OElFN192Z2dFSlZvb05jN0hXeEt0dXpTZWpOZ3BhLVdqOUx2M3NFX3c?oc=5</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>7</v>
+      </c>
+      <c r="G193" s="2" t="n">
+        <v>46014.90625</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Revolution at sea: How AI, electrification, and autonomy are transforming shipping - safety4sea</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 12:39:29 GMT</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNMWUxZkNQOFQ2MmxKNVQ5YWhRWGNHWGV3YUNyXzE0djd1blBOTVY3bjVhLVVfblo0c2ZQbjBIZk1KcncySWFDU09iQl9HcDFpakh4bHA3VXdsNzdxaFIzUmJsbG1xTnlEbjdQdW13UGozLVF5MlpyamZuODk3VzhxbkpNRG5UWm1wSTBENGE3TGdXSHJVQ05HaUtzN0NHRjNUUC0zbG1zNFdkZw?oc=5</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>7</v>
+      </c>
+      <c r="G194" s="2" t="n">
+        <v>46014.52741898148</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Google's year in review: 8 areas with research breakthroughs in 2025 - blog.google</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 17:18:57 GMT</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9HUHhmaWlhdHZXZU1JanR6TUpZNEE2dV9KQ0ZCSl8xTXhESmt0YnlISUstWVVGWEE5bEN2ZXFIckNHcVNfbzFrTlFWdVEwWDNGVEhHYzdzUUZMMjFwUkJ1dE9HNHFvR1JaRTlPZXBHZw?oc=5</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>7</v>
+      </c>
+      <c r="G195" s="2" t="n">
+        <v>46014.72149305556</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>CISA loses key employee behind early ransomware warnings - Cybersecurity Dive</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:50:46 GMT</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOUmZpbFF6QUpRMHFMU2pQMXJ6U2hweG4yTEhVNlRBME1Pb2EySldCX2NPSDNFTG1JOTM4QkVqRE9JdDBPNmlSZGxqWWN4SkRxNmx5dUZEdDFzTV91WDZnbmJSN0VERllHNjNwZ3JaVDBYVVdIWGxjM0Z1QUpmYi1wakJwQXpjZVF3eXdVZUZwMzZJTnhLdDBlRXI1N1k?oc=5</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>7</v>
+      </c>
+      <c r="G196" s="2" t="n">
+        <v>46014.66025462963</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Memory Chip Makers Say AI Alters Boom-and-Bust Cycle - Bloomberg.com</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Wed, 24 Dec 2025 01:34:56 GMT</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPTzNpWk1Ub0NEV3VKTnkwTXFTeEdLTlRkbnprTEFNUTNEXzh3MXZtcUZ1bnNyVkQ1eXJMRTc3Qm1nMXFHUUJ5TWhzRm95dFZ3Wkt3dU05eHc2a0NabnF5eUkyUWJnS0VaNDJRS2JhNHVQZWh3NXg3ZVlzVDdWcmhBc0Q0M2JKTmZQR0FjLV9meDRKMU1Db0lqNDJnMDhTUGxoUzh2TGxTc0d4Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>7</v>
+      </c>
+      <c r="G197" s="2" t="n">
+        <v>46015.06592592593</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>